<commit_message>
Updated Graphs for Sorting Programs
</commit_message>
<xml_diff>
--- a/LAB PROGRAM 3/mergesortgraph.xlsx
+++ b/LAB PROGRAM 3/mergesortgraph.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BMSCECSE-L4\Desktop\1BF24CS006\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sbisi\Desktop\Code Park\ADA-LAB\LAB PROGRAM 3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EFF0F6F5-B245-4EDC-B4EF-9ABBAB13B25A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDF02ACD-4BA6-4AA9-92A6-8C72A019EFFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F9B9998C-B9B3-4D3F-82EA-1B56B368550B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{F9B9998C-B9B3-4D3F-82EA-1B56B368550B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -118,6 +118,35 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-IN"/>
+              <a:t>Merge</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-IN" baseline="0"/>
+              <a:t> Sort Graph</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -150,25 +179,25 @@
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
-      <c:scatterChart>
-        <c:scatterStyle val="smoothMarker"/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
         <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$A$1</c:f>
+              <c:f>Sheet1!$B$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Input Size</c:v>
+                  <c:v>Time taken</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:ln w="19050" cap="rnd">
+            <a:ln w="28575" cap="rnd">
               <a:solidFill>
                 <a:schemeClr val="accent1"/>
               </a:solidFill>
@@ -177,19 +206,7 @@
             <a:effectLst/>
           </c:spPr>
           <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
+            <c:symbol val="none"/>
           </c:marker>
           <c:dLbls>
             <c:spPr>
@@ -249,154 +266,65 @@
               </c:ext>
             </c:extLst>
           </c:dLbls>
-          <c:yVal>
-            <c:numRef>
-              <c:f>Sheet1!$A$2:$A$12</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
-                <c:pt idx="0">
-                  <c:v>10000</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>20000</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>30000</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>40000</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>50000</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>60000</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>70000</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>80000</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>90000</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>100000</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="1"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-6A71-4E3B-9AF5-0C1F0992D4FA}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$B$1</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Time taken</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent2"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
+          <c:trendline>
             <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent2"/>
-              </a:solidFill>
-              <a:ln w="9525">
+              <a:ln w="19050" cap="rnd">
                 <a:solidFill>
-                  <a:schemeClr val="accent2"/>
+                  <a:schemeClr val="accent1"/>
                 </a:solidFill>
+                <a:prstDash val="sysDot"/>
               </a:ln>
               <a:effectLst/>
             </c:spPr>
-          </c:marker>
-          <c:dLbls>
-            <c:spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                <a:spAutoFit/>
-              </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="75000"/>
-                        <a:lumOff val="25000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
-            <c:dLblPos val="t"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-            <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:round/>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
-              </c:ext>
-            </c:extLst>
-          </c:dLbls>
-          <c:yVal>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$B$2:$B$12</c:f>
+              <c:f>Sheet1!$A$2:$A$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>10000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>20000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>30000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>40000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>50000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>60000</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>70000</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>80000</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>90000</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>100000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$B$2:$B$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
                 <c:pt idx="0">
                   <c:v>1E-3</c:v>
                 </c:pt>
@@ -429,120 +357,11 @@
                 </c:pt>
               </c:numCache>
             </c:numRef>
-          </c:yVal>
-          <c:smooth val="1"/>
+          </c:val>
+          <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-6A71-4E3B-9AF5-0C1F0992D4FA}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$C$1</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent3"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent3"/>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent3"/>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:dLbls>
-            <c:spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                <a:spAutoFit/>
-              </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="75000"/>
-                        <a:lumOff val="25000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
-            <c:dLblPos val="t"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-            <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:round/>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
-              </c:ext>
-            </c:extLst>
-          </c:dLbls>
-          <c:yVal>
-            <c:numRef>
-              <c:f>Sheet1!$C$2:$C$12</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="1"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-6A71-4E3B-9AF5-0C1F0992D4FA}"/>
+              <c16:uniqueId val="{00000000-A0A1-4D7D-B499-25BB31B9C7C3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -555,30 +374,17 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="1507548128"/>
-        <c:axId val="1507556032"/>
-      </c:scatterChart>
-      <c:valAx>
-        <c:axId val="1507548128"/>
+        <c:smooth val="0"/>
+        <c:axId val="2043336016"/>
+        <c:axId val="2043352816"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="2043336016"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:delete val="1"/>
+        <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
         <c:title>
           <c:tx>
             <c:rich>
@@ -600,7 +406,7 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="en-IN"/>
-                  <a:t>Time taken</a:t>
+                  <a:t>Input Size</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -634,15 +440,52 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:majorTickMark val="out"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1507556032"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2043352816"/>
         <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
       <c:valAx>
-        <c:axId val="1507556032"/>
+        <c:axId val="2043352816"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -683,7 +526,7 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="en-IN"/>
-                  <a:t>Input Size</a:t>
+                  <a:t>Time Taken</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -718,19 +561,13 @@
           </c:txPr>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
+        <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
+          <a:ln>
+            <a:noFill/>
           </a:ln>
           <a:effectLst/>
         </c:spPr>
@@ -754,9 +591,9 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1507548128"/>
+        <c:crossAx val="2043336016"/>
         <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
+        <c:crossBetween val="between"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -766,46 +603,8 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
-    <c:legend>
-      <c:legendPos val="r"/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
     <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
@@ -882,7 +681,7 @@
 </file>
 
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
@@ -909,8 +708,8 @@
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -990,6 +789,11 @@
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
   </cs:dataPoint>
   <cs:dataPoint3D>
     <cs:lnRef idx="0"/>
@@ -1000,6 +804,11 @@
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
   </cs:dataPoint3D>
   <cs:dataPointLine>
     <cs:lnRef idx="0">
@@ -1011,7 +820,7 @@
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="19050" cap="rnd">
+      <a:ln w="28575" cap="rnd">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
@@ -1031,6 +840,9 @@
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
       <a:ln w="9525">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1043,10 +855,10 @@
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="rnd">
@@ -1086,23 +898,22 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
         <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
         </a:schemeClr>
       </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
           <a:schemeClr val="tx1">
             <a:lumMod val="65000"/>
             <a:lumOff val="35000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:downBar>
@@ -1207,8 +1018,8 @@
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -1340,20 +1151,19 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
         <a:schemeClr val="lt1"/>
       </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:upBar>
@@ -1367,17 +1177,6 @@
         <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:valueAxis>
   <cs:wall>
@@ -1401,23 +1200,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>228601</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>14287</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>502046</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>43922</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>304801</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>205713</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>8997</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Chart 3">
+        <xdr:cNvPr id="5" name="Chart 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{452F422F-4EFE-4CAA-8C3B-09FBFFF194A8}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{358FA56D-FC89-15BC-7415-1297EA51D8EF}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1450,9 +1249,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1490,7 +1289,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1596,7 +1395,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1738,7 +1537,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1747,13 +1546,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14D54E98-FB01-4F7B-B813-9EB10F8B053B}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.5703125" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" customWidth="1"/>
+    <col min="1" max="1" width="16.54296875" customWidth="1"/>
+    <col min="2" max="2" width="18.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1761,7 +1560,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>10000</v>
       </c>
@@ -1769,7 +1568,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>20000</v>
       </c>
@@ -1777,7 +1576,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>30000</v>
       </c>
@@ -1785,7 +1584,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>40000</v>
       </c>
@@ -1793,7 +1592,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>50000</v>
       </c>
@@ -1801,7 +1600,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>60000</v>
       </c>
@@ -1809,7 +1608,7 @@
         <v>5.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>70000</v>
       </c>
@@ -1817,7 +1616,7 @@
         <v>6.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>80000</v>
       </c>
@@ -1825,7 +1624,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>90000</v>
       </c>
@@ -1833,7 +1632,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>100000</v>
       </c>

</xml_diff>